<commit_message>
add some features of the bulk uploads
</commit_message>
<xml_diff>
--- a/public/assets/admin_products_demo.xlsx
+++ b/public/assets/admin_products_demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\eramo-multi-vendor\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53CE3378-5F71-4576-9C84-787202763EB3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24738F3-0406-4AD1-BD10-9783AD1273C6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="100">
   <si>
     <t>id</t>
   </si>
@@ -42,9 +42,6 @@
     <t>sku</t>
   </si>
   <si>
-    <t>points</t>
-  </si>
-  <si>
     <t>description_en</t>
   </si>
   <si>
@@ -57,18 +54,6 @@
     <t>meta_title_ar</t>
   </si>
   <si>
-    <t>keywords_en</t>
-  </si>
-  <si>
-    <t>keywords_ar</t>
-  </si>
-  <si>
-    <t>details_en</t>
-  </si>
-  <si>
-    <t>details_ar</t>
-  </si>
-  <si>
     <t>summary_en</t>
   </si>
   <si>
@@ -120,30 +105,12 @@
     <t>Meta Title EN</t>
   </si>
   <si>
-    <t>Meta Title AR</t>
-  </si>
-  <si>
-    <t>keyword1, keyword2</t>
-  </si>
-  <si>
-    <t>كلمة1, كلمة2</t>
-  </si>
-  <si>
-    <t>Details EN</t>
-  </si>
-  <si>
-    <t>تفاصيل AR</t>
-  </si>
-  <si>
     <t>Summary EN</t>
   </si>
   <si>
     <t>ملخص AR</t>
   </si>
   <si>
-    <t>https://bnaia.com/storage/product-images/sample1.jpg</t>
-  </si>
-  <si>
     <t>no</t>
   </si>
   <si>
@@ -165,48 +132,15 @@
     <t>Meta Title EN 2</t>
   </si>
   <si>
-    <t>Meta Title AR 2</t>
-  </si>
-  <si>
-    <t>keyword3, keyword4</t>
-  </si>
-  <si>
-    <t>كلمة3, كلمة4</t>
-  </si>
-  <si>
-    <t>Details EN 2</t>
-  </si>
-  <si>
-    <t>تفاصيل AR 2</t>
-  </si>
-  <si>
     <t>Summary EN 2</t>
   </si>
   <si>
     <t>ملخص AR 2</t>
   </si>
   <si>
-    <t>https://bnaia.com/storage/product-images/sample2.jpg</t>
-  </si>
-  <si>
     <t>product_id</t>
   </si>
   <si>
-    <t>https://bnaia.com/storage/product-images/sample1-1.jpg</t>
-  </si>
-  <si>
-    <t>https://bnaia.com/storage/product-images/sample1-2.jpg</t>
-  </si>
-  <si>
-    <t>https://bnaia.com/storage/product-images/sample2-1.jpg</t>
-  </si>
-  <si>
-    <t>variant_id</t>
-  </si>
-  <si>
-    <t>variants_configuration_id</t>
-  </si>
-  <si>
     <t>price</t>
   </si>
   <si>
@@ -228,12 +162,6 @@
     <t>name_ar</t>
   </si>
   <si>
-    <t>subtitle_en</t>
-  </si>
-  <si>
-    <t>subtitle_ar</t>
-  </si>
-  <si>
     <t>start_date</t>
   </si>
   <si>
@@ -258,21 +186,6 @@
     <t>لفترة محدودة</t>
   </si>
   <si>
-    <t>Occasion description EN</t>
-  </si>
-  <si>
-    <t>وصف المناسبة AR</t>
-  </si>
-  <si>
-    <t>https://bnaia.com/storage/occasions/ramadan.jpg</t>
-  </si>
-  <si>
-    <t>2026-03-01</t>
-  </si>
-  <si>
-    <t>2026-03-31</t>
-  </si>
-  <si>
     <t>Eid Offers</t>
   </si>
   <si>
@@ -291,39 +204,154 @@
     <t>حتى نفاذ الكمية</t>
   </si>
   <si>
-    <t>Another occasion description EN</t>
-  </si>
-  <si>
-    <t>https://bnaia.com/storage/occasions/eid.jpg</t>
-  </si>
-  <si>
-    <t>2026-04-01</t>
-  </si>
-  <si>
-    <t>2026-04-10</t>
-  </si>
-  <si>
     <t>occasion_id</t>
   </si>
   <si>
-    <t>product_size_color_id</t>
-  </si>
-  <si>
     <t>special_price</t>
   </si>
   <si>
     <t>position</t>
+  </si>
+  <si>
+    <t>vendor_id</t>
+  </si>
+  <si>
+    <t>features_en</t>
+  </si>
+  <si>
+    <t>features_ar</t>
+  </si>
+  <si>
+    <t>features en</t>
+  </si>
+  <si>
+    <t>فيتشر عربى</t>
+  </si>
+  <si>
+    <t>instructions_en</t>
+  </si>
+  <si>
+    <t>instructions_ar</t>
+  </si>
+  <si>
+    <t>instructions en</t>
+  </si>
+  <si>
+    <t>انستراكشنز عربى</t>
+  </si>
+  <si>
+    <t>extra_description_en</t>
+  </si>
+  <si>
+    <t>extra_description_ar</t>
+  </si>
+  <si>
+    <t>extra description en</t>
+  </si>
+  <si>
+    <t>اكسترا ديسكريبشن عربى</t>
+  </si>
+  <si>
+    <t>material_en</t>
+  </si>
+  <si>
+    <t>material_ar</t>
+  </si>
+  <si>
+    <t>material en</t>
+  </si>
+  <si>
+    <t>ماتييريال عربي</t>
+  </si>
+  <si>
+    <t>ميتا عربي</t>
+  </si>
+  <si>
+    <t>meta_description_en</t>
+  </si>
+  <si>
+    <t>meta_description_ar</t>
+  </si>
+  <si>
+    <t>meta description en</t>
+  </si>
+  <si>
+    <t>ميتا ديسكريبشن عربي</t>
+  </si>
+  <si>
+    <t>meta_keywords_en</t>
+  </si>
+  <si>
+    <t>meta_keywords_ar</t>
+  </si>
+  <si>
+    <t>max_per_order</t>
+  </si>
+  <si>
+    <t>https://bnaia.com/dashboards/img/logo.png</t>
+  </si>
+  <si>
+    <t>is_main</t>
+  </si>
+  <si>
+    <t>variant_configuration_id</t>
+  </si>
+  <si>
+    <t>variant_sku</t>
+  </si>
+  <si>
+    <t>sub_title_en</t>
+  </si>
+  <si>
+    <t>sub_title_ar</t>
+  </si>
+  <si>
+    <t>meta title en</t>
+  </si>
+  <si>
+    <t>ميتا تيتل عربي</t>
+  </si>
+  <si>
+    <t>first-second-third</t>
+  </si>
+  <si>
+    <t>اول-ثانى-ثالث</t>
+  </si>
+  <si>
+    <t>is_active</t>
+  </si>
+  <si>
+    <t>keyword1-keyword2</t>
+  </si>
+  <si>
+    <t>كلمة1-كلمة2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -343,13 +371,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -652,357 +687,418 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="12" width="24.21875" customWidth="1"/>
+    <col min="13" max="21" width="24.88671875" customWidth="1"/>
+    <col min="22" max="31" width="24.21875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="I1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="K1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="L1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="V1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="W1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
+      <c r="X1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="AC1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="AD1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="AE1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" t="s">
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="I2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" t="s">
+      <c r="J2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="K2" t="s">
         <v>24</v>
       </c>
-      <c r="C2" t="s">
+      <c r="L2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="V2" t="s">
         <v>25</v>
       </c>
-      <c r="D2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2" t="s">
-        <v>29</v>
-      </c>
-      <c r="I2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M2" t="s">
-        <v>34</v>
-      </c>
-      <c r="N2" t="s">
-        <v>35</v>
-      </c>
-      <c r="O2" t="s">
-        <v>36</v>
-      </c>
-      <c r="P2" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q2">
-        <v>1</v>
-      </c>
-      <c r="S2">
-        <v>1</v>
-      </c>
-      <c r="T2">
-        <v>1</v>
-      </c>
-      <c r="U2">
-        <v>1</v>
-      </c>
-      <c r="V2">
-        <v>1</v>
-      </c>
-      <c r="W2">
-        <v>50</v>
-      </c>
-      <c r="X2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="W2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>99</v>
+      </c>
+      <c r="AB2">
+        <v>1</v>
+      </c>
+      <c r="AC2">
+        <v>1</v>
+      </c>
+      <c r="AD2">
+        <v>1</v>
+      </c>
+      <c r="AE2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>43</v>
+      <c r="B3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="1">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
       </c>
       <c r="H3" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="I3" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="J3" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="K3" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="L3" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="M3" t="s">
-        <v>49</v>
-      </c>
-      <c r="N3" t="s">
-        <v>50</v>
-      </c>
-      <c r="O3" t="s">
-        <v>51</v>
-      </c>
-      <c r="P3" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q3">
-        <v>1</v>
-      </c>
-      <c r="R3">
-        <v>1</v>
-      </c>
-      <c r="S3">
+        <v>36</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="V3" t="s">
+        <v>34</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>99</v>
+      </c>
+      <c r="AB3">
         <v>2</v>
       </c>
-      <c r="T3">
+      <c r="AC3">
         <v>3</v>
       </c>
-      <c r="U3">
+      <c r="AD3">
         <v>4</v>
       </c>
-      <c r="V3">
+      <c r="AE3">
         <v>2</v>
-      </c>
-      <c r="W3">
-        <v>75</v>
-      </c>
-      <c r="X3" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.5546875" customWidth="1"/>
+    <col min="2" max="2" width="75" customWidth="1"/>
+    <col min="3" max="3" width="56.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>57</v>
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{4A0E61C4-73F4-4C4B-B42C-470C6E232075}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{A3B5C720-B885-4284-94A2-CB22F333273E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="4" width="25.5546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>299</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>61</v>
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2">
+        <v>101</v>
       </c>
       <c r="D2">
-        <v>101</v>
-      </c>
-      <c r="E2">
-        <v>20</v>
-      </c>
-      <c r="F2">
         <v>199.99</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>298</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>62</v>
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3">
+        <v>102</v>
       </c>
       <c r="D3">
-        <v>102</v>
-      </c>
-      <c r="E3">
-        <v>30</v>
-      </c>
-      <c r="F3">
         <v>209.99</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>297</v>
-      </c>
-      <c r="B4">
         <v>2</v>
       </c>
-      <c r="C4" t="s">
-        <v>63</v>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4">
+        <v>103</v>
       </c>
       <c r="D4">
-        <v>103</v>
-      </c>
-      <c r="E4">
-        <v>40</v>
-      </c>
-      <c r="F4">
         <v>299.99</v>
       </c>
     </row>
@@ -1015,16 +1111,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="3" width="33.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C1" t="s">
-        <v>22</v>
+      <c r="A1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -1067,18 +1166,25 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="13" width="20.6640625" customWidth="1"/>
+    <col min="14" max="15" width="20.6640625" style="4" customWidth="1"/>
+    <col min="16" max="16" width="38" style="4" customWidth="1"/>
+    <col min="17" max="17" width="24.5546875" customWidth="1"/>
+    <col min="18" max="24" width="20.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="C1" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -1086,146 +1192,195 @@
       <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K1" t="s">
-        <v>69</v>
-      </c>
-      <c r="L1" t="s">
-        <v>70</v>
-      </c>
-      <c r="M1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="E2" t="s">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="F2" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="G2" t="s">
-        <v>76</v>
-      </c>
-      <c r="H2" t="s">
-        <v>77</v>
-      </c>
-      <c r="I2" t="s">
-        <v>78</v>
-      </c>
-      <c r="J2" t="s">
-        <v>79</v>
-      </c>
-      <c r="K2" t="s">
-        <v>80</v>
-      </c>
-      <c r="L2" t="s">
-        <v>81</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N2" s="3">
+        <v>45785</v>
+      </c>
+      <c r="O2" s="3">
+        <v>45785</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C3" t="s">
+      <c r="K3" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" t="s">
-        <v>86</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="L3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N3" s="3">
+        <v>45785</v>
+      </c>
+      <c r="O3" s="3">
+        <v>45785</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="H3" t="s">
-        <v>88</v>
-      </c>
-      <c r="I3" t="s">
-        <v>44</v>
-      </c>
-      <c r="J3" t="s">
-        <v>89</v>
-      </c>
-      <c r="K3" t="s">
-        <v>90</v>
-      </c>
-      <c r="L3" t="s">
-        <v>91</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
+      <c r="Q3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="P2" r:id="rId1" xr:uid="{0564E689-CD70-4D38-A606-A8CDA61D4258}"/>
+    <hyperlink ref="P3" r:id="rId2" xr:uid="{F599F08E-1F0B-4AE5-8F82-29182A0B2314}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="5" width="43.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B1" t="s">
-        <v>93</v>
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>60</v>
       </c>
       <c r="E1" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>299</v>
+      <c r="B2" t="s">
+        <v>39</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -1241,8 +1396,8 @@
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3">
-        <v>298</v>
+      <c r="B3" t="s">
+        <v>39</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -1252,20 +1407,6 @@
       </c>
       <c r="E3">
         <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4">
-        <v>297</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>